<commit_message>
Fix test data and add balance sheet/cash flow calculation rules
- Reduced Cost of Sales from 70% to 55% of revenue so EBITDA is positive
  (~18% margin), realistic for a PE logistics company
- Added 30+ label mappings covering balance sheet and cash flow line items
- Added 11 new calculation rules for balance sheet and cash flow totals
- Updated test assertions to match new financial data

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/testdata/NorthStar_Logistics_Feb2026.xlsx
+++ b/testdata/NorthStar_Logistics_Feb2026.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,11 +30,6 @@
     </font>
     <font>
       <b val="1"/>
-      <sz val="14"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <sz val="12"/>
     </font>
   </fonts>
   <fills count="2">
@@ -57,11 +52,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -430,45 +423,45 @@
   <dimension ref="A1:D21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="32" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="35" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>NorthStar Logistics Ltd</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr"/>
-      <c r="C1" s="1" t="inlineStr"/>
-      <c r="D1" s="1" t="inlineStr"/>
+      <c r="B1" t="inlineStr"/>
+      <c r="C1" t="inlineStr"/>
+      <c r="D1" t="inlineStr"/>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>Profit &amp; Loss Summary — February 2026</t>
         </is>
       </c>
-      <c r="B2" s="1" t="inlineStr"/>
-      <c r="C2" s="1" t="inlineStr"/>
-      <c r="D2" s="1" t="inlineStr"/>
+      <c r="B2" t="inlineStr"/>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr"/>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="A3" s="1" t="inlineStr"/>
+      <c r="B3" s="1" t="inlineStr">
         <is>
           <t>Feb 2026</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" s="1" t="inlineStr">
         <is>
           <t>Jan 2026</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D3" s="1" t="inlineStr">
         <is>
           <t>Feb 2025</t>
         </is>
@@ -480,13 +473,13 @@
           <t>Net Sales</t>
         </is>
       </c>
-      <c r="B4" s="3" t="n">
+      <c r="B4" t="n">
         <v>2609250</v>
       </c>
-      <c r="C4" s="3" t="n">
+      <c r="C4" t="n">
         <v>2450000</v>
       </c>
-      <c r="D4" s="3" t="n">
+      <c r="D4" t="n">
         <v>2280000</v>
       </c>
     </row>
@@ -496,18 +489,18 @@
           <t>Cost of Sales</t>
         </is>
       </c>
-      <c r="B5" s="3" t="n">
-        <v>-1852000</v>
-      </c>
-      <c r="C5" s="3" t="n">
-        <v>-1715000</v>
-      </c>
-      <c r="D5" s="3" t="n">
-        <v>-1596000</v>
+      <c r="B5" t="n">
+        <v>-1435088</v>
+      </c>
+      <c r="C5" t="n">
+        <v>-1347500</v>
+      </c>
+      <c r="D5" t="n">
+        <v>-1254000</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="1" t="inlineStr">
         <is>
           <t>Gross Profit</t>
         </is>
@@ -519,14 +512,14 @@
           <t>Warehouse &amp; Distribution</t>
         </is>
       </c>
-      <c r="B7" s="3" t="n">
-        <v>-260900</v>
-      </c>
-      <c r="C7" s="3" t="n">
-        <v>-245000</v>
-      </c>
-      <c r="D7" s="3" t="n">
-        <v>-228000</v>
+      <c r="B7" t="n">
+        <v>-182648</v>
+      </c>
+      <c r="C7" t="n">
+        <v>-171500</v>
+      </c>
+      <c r="D7" t="n">
+        <v>-159600</v>
       </c>
     </row>
     <row r="8">
@@ -535,14 +528,14 @@
           <t>Fleet Operating Costs</t>
         </is>
       </c>
-      <c r="B8" s="3" t="n">
-        <v>-149450</v>
-      </c>
-      <c r="C8" s="3" t="n">
-        <v>-122500</v>
-      </c>
-      <c r="D8" s="3" t="n">
-        <v>-114000</v>
+      <c r="B8" t="n">
+        <v>-104770</v>
+      </c>
+      <c r="C8" t="n">
+        <v>-85750</v>
+      </c>
+      <c r="D8" t="n">
+        <v>-79800</v>
       </c>
     </row>
     <row r="9">
@@ -551,14 +544,14 @@
           <t>Staff Costs</t>
         </is>
       </c>
-      <c r="B9" s="3" t="n">
-        <v>-382200</v>
-      </c>
-      <c r="C9" s="3" t="n">
-        <v>-367500</v>
-      </c>
-      <c r="D9" s="3" t="n">
-        <v>-342000</v>
+      <c r="B9" t="n">
+        <v>-313110</v>
+      </c>
+      <c r="C9" t="n">
+        <v>-294000</v>
+      </c>
+      <c r="D9" t="n">
+        <v>-273600</v>
       </c>
     </row>
     <row r="10">
@@ -567,14 +560,14 @@
           <t>Premises</t>
         </is>
       </c>
-      <c r="B10" s="3" t="n">
-        <v>-75000</v>
-      </c>
-      <c r="C10" s="3" t="n">
-        <v>-73500</v>
-      </c>
-      <c r="D10" s="3" t="n">
-        <v>-66000</v>
+      <c r="B10" t="n">
+        <v>-54794</v>
+      </c>
+      <c r="C10" t="n">
+        <v>-51450</v>
+      </c>
+      <c r="D10" t="n">
+        <v>-47880</v>
       </c>
     </row>
     <row r="11">
@@ -583,14 +576,14 @@
           <t>Professional Fees</t>
         </is>
       </c>
-      <c r="B11" s="3" t="n">
-        <v>-9800</v>
-      </c>
-      <c r="C11" s="3" t="n">
-        <v>-24500</v>
-      </c>
-      <c r="D11" s="3" t="n">
-        <v>-22800</v>
+      <c r="B11" t="n">
+        <v>-6850</v>
+      </c>
+      <c r="C11" t="n">
+        <v>-17150</v>
+      </c>
+      <c r="D11" t="n">
+        <v>-15960</v>
       </c>
     </row>
     <row r="12">
@@ -599,25 +592,25 @@
           <t>Other Overheads</t>
         </is>
       </c>
-      <c r="B12" s="3" t="n">
-        <v>-52200</v>
-      </c>
-      <c r="C12" s="3" t="n">
-        <v>-49000</v>
-      </c>
-      <c r="D12" s="3" t="n">
-        <v>-45600</v>
+      <c r="B12" t="n">
+        <v>-36530</v>
+      </c>
+      <c r="C12" t="n">
+        <v>-34300</v>
+      </c>
+      <c r="D12" t="n">
+        <v>-31920</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="1" t="inlineStr">
         <is>
           <t>Total Overheads</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="1" t="inlineStr">
         <is>
           <t>Operating Profit Before D&amp;A</t>
         </is>
@@ -629,13 +622,13 @@
           <t>Depreciation</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n">
+      <c r="B15" t="n">
         <v>-65250</v>
       </c>
-      <c r="C15" s="3" t="n">
+      <c r="C15" t="n">
         <v>-61250</v>
       </c>
-      <c r="D15" s="3" t="n">
+      <c r="D15" t="n">
         <v>-57000</v>
       </c>
     </row>
@@ -645,18 +638,18 @@
           <t>Amortisation</t>
         </is>
       </c>
-      <c r="B16" s="3" t="n">
+      <c r="B16" t="n">
         <v>-13050</v>
       </c>
-      <c r="C16" s="3" t="n">
+      <c r="C16" t="n">
         <v>-12250</v>
       </c>
-      <c r="D16" s="3" t="n">
+      <c r="D16" t="n">
         <v>-11400</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="1" t="inlineStr">
         <is>
           <t>Operating Profit</t>
         </is>
@@ -668,32 +661,32 @@
           <t>Interest Payable</t>
         </is>
       </c>
-      <c r="B18" s="3" t="n">
+      <c r="B18" t="n">
         <v>-19575</v>
       </c>
-      <c r="C18" s="3" t="n">
+      <c r="C18" t="n">
         <v>-18375</v>
       </c>
-      <c r="D18" s="3" t="n">
+      <c r="D18" t="n">
         <v>-17100</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19" s="1" t="inlineStr">
         <is>
           <t>Profit Before Tax</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="A20" s="1" t="inlineStr">
         <is>
           <t>Tax</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
+      <c r="A21" s="1" t="inlineStr">
         <is>
           <t>Net Profit</t>
         </is>
@@ -713,41 +706,42 @@
   <dimension ref="A1:B24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="32" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="35" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>NorthStar Logistics Ltd</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr"/>
+      <c r="B1" t="inlineStr"/>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>Balance Sheet as at 28 February 2026</t>
         </is>
       </c>
-      <c r="B2" s="1" t="inlineStr"/>
+      <c r="B2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr"/>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="A3" t="inlineStr"/>
+      <c r="B3" s="1" t="inlineStr">
         <is>
           <t>Feb 2026</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="1" t="inlineStr">
         <is>
           <t>FIXED ASSETS</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -770,19 +764,18 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="1" t="inlineStr">
         <is>
           <t>Total Fixed Assets</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="1" t="inlineStr">
         <is>
           <t>CURRENT ASSETS</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -825,19 +818,18 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="1" t="inlineStr">
         <is>
           <t>Total Current Assets</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="1" t="inlineStr">
         <is>
           <t>CURRENT LIABILITIES</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -870,33 +862,32 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="1" t="inlineStr">
         <is>
           <t>Total Current Liabilities</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19" s="1" t="inlineStr">
         <is>
           <t>Net Current Assets</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="A20" s="1" t="inlineStr">
         <is>
           <t>NET ASSETS</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
+      <c r="A21" s="1" t="inlineStr">
         <is>
           <t>EQUITY</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -909,14 +900,14 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
+      <c r="A23" s="1" t="inlineStr">
         <is>
           <t>Retained Earnings</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
+      <c r="A24" s="1" t="inlineStr">
         <is>
           <t>Total Equity</t>
         </is>
@@ -936,41 +927,42 @@
   <dimension ref="A1:B23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="38" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="35" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>NorthStar Logistics Ltd</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr"/>
+      <c r="B1" t="inlineStr"/>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>Cash Flow Statement — February 2026</t>
         </is>
       </c>
-      <c r="B2" s="1" t="inlineStr"/>
+      <c r="B2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr"/>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="A3" t="inlineStr"/>
+      <c r="B3" s="1" t="inlineStr">
         <is>
           <t>Feb 2026</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="1" t="inlineStr">
         <is>
           <t>OPERATING ACTIVITIES</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1023,7 +1015,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="1" t="inlineStr">
         <is>
           <t>Cash from Operations</t>
         </is>
@@ -1040,19 +1032,18 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="1" t="inlineStr">
         <is>
           <t>Net Cash from Operating</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="1" t="inlineStr">
         <is>
           <t>INVESTING ACTIVITIES</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1075,19 +1066,18 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" s="1" t="inlineStr">
         <is>
           <t>Net Cash from Investing</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="1" t="inlineStr">
         <is>
           <t>FINANCING ACTIVITIES</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1110,14 +1100,14 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="A20" s="1" t="inlineStr">
         <is>
           <t>Net Cash from Financing</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
+      <c r="A21" s="1" t="inlineStr">
         <is>
           <t>Net Change in Cash</t>
         </is>
@@ -1134,7 +1124,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
+      <c r="A23" s="1" t="inlineStr">
         <is>
           <t>Closing Cash Balance</t>
         </is>
@@ -1154,41 +1144,42 @@
   <dimension ref="A1:C12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="35" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Key Performance Indicators</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr"/>
-      <c r="C1" s="1" t="inlineStr"/>
+      <c r="B1" t="inlineStr"/>
+      <c r="C1" t="inlineStr"/>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>February 2026</t>
         </is>
       </c>
-      <c r="B2" s="1" t="inlineStr"/>
-      <c r="C2" s="1" t="inlineStr"/>
+      <c r="B2" t="inlineStr"/>
+      <c r="C2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="1" t="inlineStr">
         <is>
           <t>Metric</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="1" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" s="1" t="inlineStr">
         <is>
           <t>Prior Month</t>
         </is>

</xml_diff>

<commit_message>
Extend calculation layer to BrightPath (CSV) and Helix (PDF), add upload form
- Fix calculator to handle CSV parser output: NaN→None, --- separators
  don't reset headers, nan cells treated as blank for injection
- Add BrightPath label mappings (11) and calculation rules (3) to seed_data
- Create Helix Manufacturing Q4 2025 PDF with blank formula rows
- Add Helix label mappings (14) and calculation rules (4) to seed_data
- Build upload form page (upload.html) with drag-drop, progress, auto-process
- Update test data: BrightPath CSV blanked formula rows, NorthStar Excel
  reconciled CF with BS
- Add 17 new tests (NaN handling, BrightPath integration, Helix integration)
- Update pre-existing tests for new test data values
- 142 tests passing

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/testdata/NorthStar_Logistics_Feb2026.xlsx
+++ b/testdata/NorthStar_Logistics_Feb2026.xlsx
@@ -784,7 +784,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>380000</v>
+        <v>422500</v>
       </c>
     </row>
     <row r="10">
@@ -794,7 +794,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>652000</v>
+        <v>764500</v>
       </c>
     </row>
     <row r="11">
@@ -838,7 +838,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>-510000</v>
+        <v>-344240</v>
       </c>
     </row>
     <row r="16">
@@ -971,7 +971,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>79825</v>
+        <v>397160</v>
       </c>
     </row>
     <row r="6">
@@ -991,7 +991,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>-39500</v>
+        <v>-152000</v>
       </c>
     </row>
     <row r="8">
@@ -1001,7 +1001,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>-12500</v>
+        <v>-55000</v>
       </c>
     </row>
     <row r="9">
@@ -1011,7 +1011,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>25500</v>
+        <v>-145760</v>
       </c>
     </row>
     <row r="10">

</xml_diff>